<commit_message>
Schematic & LTspice changes - changes made recorded in onenote
</commit_message>
<xml_diff>
--- a/Meeting_Minutes(TemporarilyHere)/InterfacePowerDesign.xlsx
+++ b/Meeting_Minutes(TemporarilyHere)/InterfacePowerDesign.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\seong\Bachelor_Thesis\uz_per_wolfspeed_25kw_FM3\Meeting_Minutes(TemporarilyHere)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEB69769-EB5F-4916-90C1-48A584CEE186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C88AA39-E049-4F82-83D9-3730A15CA9FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="61">
   <si>
     <t>Voltage Level</t>
   </si>
@@ -162,9 +162,6 @@
     <t>775uA</t>
   </si>
   <si>
-    <t>6.9mA</t>
-  </si>
-  <si>
     <t>2.5mA</t>
   </si>
   <si>
@@ -190,6 +187,50 @@
   </si>
   <si>
     <t>max 16mA</t>
+  </si>
+  <si>
+    <t>max. 80mA (continuous forward current I_Fdc)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">High Level Supply Current: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>max 6.3mA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> at 5.25Vcc</t>
+    </r>
+  </si>
+  <si>
+    <t>max 16mA -&gt; high level output current at V_cc =3V</t>
+  </si>
+  <si>
+    <t>I_cc max 10 uA</t>
+  </si>
+  <si>
+    <t>2mA</t>
+  </si>
+  <si>
+    <t>33mA Transmitter + inverter</t>
+  </si>
+  <si>
+    <t>10mA</t>
   </si>
 </sst>
 </file>
@@ -227,7 +268,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -250,11 +291,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -262,6 +340,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -278,6 +375,99 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>232410</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>114262</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3CECE3FD-2BC3-3526-E52F-F17221ED5C24}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7993380" y="5486400"/>
+          <a:ext cx="4072890" cy="2125942"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>397437</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>187393</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>88007</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A35E5FAB-75F9-F8DC-6755-1DB9846737F3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10953750" y="2409117"/>
+          <a:ext cx="5548063" cy="2982410"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -543,7 +733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:G40"/>
+  <dimension ref="A2:H40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="11.15625" bestFit="1" customWidth="1"/>
@@ -555,7 +745,7 @@
     <col min="7" max="7" width="18.7890625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -578,7 +768,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -594,10 +784,10 @@
         <v>44</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
         <v>3</v>
@@ -609,10 +799,10 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="2"/>
       <c r="B5" s="2" t="s">
         <v>3</v>
@@ -624,10 +814,10 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="2"/>
       <c r="B6" s="3" t="s">
         <v>11</v>
@@ -639,10 +829,10 @@
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
@@ -656,10 +846,10 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="2"/>
       <c r="B8" s="2" t="s">
         <v>13</v>
@@ -671,10 +861,10 @@
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
         <v>13</v>
@@ -686,10 +876,10 @@
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
         <v>13</v>
@@ -701,10 +891,10 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="2" t="s">
         <v>14</v>
       </c>
@@ -718,10 +908,10 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
         <v>15</v>
@@ -733,10 +923,10 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
         <v>15</v>
@@ -748,10 +938,10 @@
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
@@ -761,12 +951,17 @@
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+      <c r="F14" s="5" t="s">
+        <v>60</v>
+      </c>
       <c r="G14" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>50</v>
+      </c>
+      <c r="H14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
         <v>18</v>
@@ -774,12 +969,12 @@
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
+      <c r="F15" s="6"/>
       <c r="G15" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
         <v>19</v>
@@ -787,12 +982,12 @@
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+      <c r="F16" s="6"/>
       <c r="G16" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
         <v>20</v>
@@ -800,12 +995,12 @@
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
+      <c r="F17" s="6"/>
       <c r="G17" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
         <v>21</v>
@@ -813,12 +1008,12 @@
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+      <c r="F18" s="6"/>
       <c r="G18" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="2"/>
       <c r="B19" s="2" t="s">
         <v>22</v>
@@ -826,12 +1021,12 @@
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
+      <c r="F19" s="6"/>
       <c r="G19" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="2"/>
       <c r="B20" s="2" t="s">
         <v>23</v>
@@ -839,12 +1034,12 @@
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+      <c r="F20" s="7"/>
       <c r="G20" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="2"/>
       <c r="B21" s="2" t="s">
         <v>24</v>
@@ -853,13 +1048,13 @@
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="2"/>
       <c r="B22" s="2" t="s">
         <v>25</v>
@@ -869,10 +1064,13 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>53</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="2"/>
       <c r="B23" s="2" t="s">
         <v>26</v>
@@ -882,10 +1080,10 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
         <v>27</v>
@@ -895,10 +1093,10 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
       <c r="G24" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="2"/>
       <c r="B25" s="2" t="s">
         <v>28</v>
@@ -908,10 +1106,10 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="2"/>
       <c r="B26" s="2" t="s">
         <v>29</v>
@@ -921,10 +1119,10 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
         <v>30</v>
@@ -934,10 +1132,10 @@
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="2"/>
       <c r="B28" s="2" t="s">
         <v>31</v>
@@ -948,7 +1146,7 @@
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="2"/>
       <c r="B29" s="2" t="s">
         <v>32</v>
@@ -959,7 +1157,7 @@
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
         <v>33</v>
@@ -970,7 +1168,7 @@
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="2"/>
       <c r="B31" s="2" t="s">
         <v>34</v>
@@ -981,7 +1179,7 @@
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="2"/>
       <c r="B32" s="2" t="s">
         <v>35</v>
@@ -1022,9 +1220,11 @@
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
+      <c r="F35" s="8" t="s">
+        <v>59</v>
+      </c>
       <c r="G35" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -1035,9 +1235,9 @@
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
+      <c r="F36" s="9"/>
       <c r="G36" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -1048,9 +1248,9 @@
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
+      <c r="F37" s="9"/>
       <c r="G37" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -1061,9 +1261,9 @@
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
+      <c r="F38" s="10"/>
       <c r="G38" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -1076,7 +1276,7 @@
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
       <c r="G39" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -1089,11 +1289,16 @@
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
       <c r="G40" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F35:F38"/>
+    <mergeCell ref="F14:F20"/>
+  </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>